<commit_message>
Update community hub templates and JSON configuration
- Replace existing Excel templates for various community hubs with updated versions in the `public/community-hubs-templates` directory.
- Modify `devcon-7-bundle.json` to update the version number and adjust room IDs and colors for the Privacy and Onchain Art hubs, ensuring accurate representation in the event application.
</commit_message>
<xml_diff>
--- a/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
+++ b/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
@@ -95,7 +95,7 @@
       <name val="Calibri"/>
       <u val="single"/>
       <color rgb="000563C1"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="8">
@@ -657,12 +657,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>Hub name</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Agentic Hub</t>
         </is>
@@ -674,14 +669,9 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Read me</t>
-        </is>
-      </c>
-      <c r="B2" s="19" t="inlineStr">
-        <is>
-          <t>https://docs.fileverse.io/u/0/w/96dc21d9/document/hpBL2denPdQsJW89fwj3sa#k=aqZTmKgiOCX_MQFJ_IV_8fBE0ffCJCz9Hfl6PC95zUs</t>
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Read me: how to fill in this sheet</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -2519,8 +2509,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="B4:B103" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Day" error="Pick a day from the list." allowBlank="1" type="list">
@@ -2537,7 +2527,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="A2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update community hub templates and documentation for Devcon 8, including multiple Excel files and adjustments to the schedule format in the markdown documentation.
</commit_message>
<xml_diff>
--- a/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
+++ b/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ103"/>
+  <dimension ref="A1:AJ163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="36" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -662,11 +662,6 @@
           <t>Agentic Hub</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -674,11 +669,6 @@
           <t>Read me: how to fill in this sheet</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>09:10</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -724,11 +714,6 @@
       <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Topic (optional)</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>09:20</t>
         </is>
       </c>
     </row>
@@ -746,11 +731,6 @@
       <c r="G4" s="9" t="n"/>
       <c r="H4" s="9" t="n"/>
       <c r="I4" s="9" t="n"/>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
@@ -766,11 +746,6 @@
       <c r="G5" s="9" t="n"/>
       <c r="H5" s="9" t="n"/>
       <c r="I5" s="9" t="n"/>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -786,11 +761,6 @@
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>09:50</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -806,11 +776,6 @@
       <c r="G7" s="9" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -826,11 +791,6 @@
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
-      <c r="AJ8" t="inlineStr">
-        <is>
-          <t>10:10</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -846,11 +806,6 @@
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
       <c r="I9" s="9" t="n"/>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>10:20</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -866,11 +821,6 @@
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -886,11 +836,6 @@
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n"/>
       <c r="I11" s="9" t="n"/>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -906,11 +851,6 @@
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>10:50</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
@@ -926,11 +866,6 @@
       <c r="G13" s="9" t="n"/>
       <c r="H13" s="9" t="n"/>
       <c r="I13" s="9" t="n"/>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
@@ -946,11 +881,6 @@
       <c r="G14" s="9" t="n"/>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>11:10</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
@@ -966,11 +896,6 @@
       <c r="G15" s="9" t="n"/>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="9" t="n"/>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>11:20</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
@@ -986,11 +911,6 @@
       <c r="G16" s="9" t="n"/>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -1006,11 +926,6 @@
       <c r="G17" s="9" t="n"/>
       <c r="H17" s="9" t="n"/>
       <c r="I17" s="9" t="n"/>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>11:40</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
@@ -1026,11 +941,6 @@
       <c r="G18" s="9" t="n"/>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>11:50</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
@@ -1046,11 +956,6 @@
       <c r="G19" s="9" t="n"/>
       <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
@@ -1066,11 +971,6 @@
       <c r="G20" s="9" t="n"/>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
-      <c r="AJ20" t="inlineStr">
-        <is>
-          <t>12:10</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="inlineStr">
@@ -1086,11 +986,6 @@
       <c r="G21" s="9" t="n"/>
       <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
-      <c r="AJ21" t="inlineStr">
-        <is>
-          <t>12:20</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
@@ -1106,11 +1001,6 @@
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
-      <c r="AJ22" t="inlineStr">
-        <is>
-          <t>12:30</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
@@ -1126,11 +1016,6 @@
       <c r="G23" s="9" t="n"/>
       <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
-      <c r="AJ23" t="inlineStr">
-        <is>
-          <t>12:40</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -1146,11 +1031,6 @@
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
-      <c r="AJ24" t="inlineStr">
-        <is>
-          <t>12:50</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
@@ -1166,11 +1046,6 @@
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="9" t="n"/>
       <c r="I25" s="9" t="n"/>
-      <c r="AJ25" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
@@ -1186,11 +1061,6 @@
       <c r="G26" s="9" t="n"/>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
-      <c r="AJ26" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
@@ -1206,11 +1076,6 @@
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="9" t="n"/>
       <c r="I27" s="9" t="n"/>
-      <c r="AJ27" t="inlineStr">
-        <is>
-          <t>13:20</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
@@ -1226,11 +1091,6 @@
       <c r="G28" s="9" t="n"/>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
-      <c r="AJ28" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
@@ -1246,11 +1106,6 @@
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n"/>
       <c r="I29" s="9" t="n"/>
-      <c r="AJ29" t="inlineStr">
-        <is>
-          <t>13:40</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
@@ -1266,11 +1121,6 @@
       <c r="G30" s="9" t="n"/>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
-      <c r="AJ30" t="inlineStr">
-        <is>
-          <t>13:50</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
@@ -1286,11 +1136,6 @@
       <c r="G31" s="9" t="n"/>
       <c r="H31" s="9" t="n"/>
       <c r="I31" s="9" t="n"/>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
@@ -1306,11 +1151,6 @@
       <c r="G32" s="9" t="n"/>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
-      <c r="AJ32" t="inlineStr">
-        <is>
-          <t>14:10</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
@@ -1326,11 +1166,6 @@
       <c r="G33" s="9" t="n"/>
       <c r="H33" s="9" t="n"/>
       <c r="I33" s="9" t="n"/>
-      <c r="AJ33" t="inlineStr">
-        <is>
-          <t>14:20</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
@@ -1346,11 +1181,6 @@
       <c r="G34" s="9" t="n"/>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
-      <c r="AJ34" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
@@ -1366,11 +1196,6 @@
       <c r="G35" s="9" t="n"/>
       <c r="H35" s="9" t="n"/>
       <c r="I35" s="9" t="n"/>
-      <c r="AJ35" t="inlineStr">
-        <is>
-          <t>14:40</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
@@ -1386,11 +1211,6 @@
       <c r="G36" s="9" t="n"/>
       <c r="H36" s="9" t="n"/>
       <c r="I36" s="9" t="n"/>
-      <c r="AJ36" t="inlineStr">
-        <is>
-          <t>14:50</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
@@ -1406,11 +1226,6 @@
       <c r="G37" s="9" t="n"/>
       <c r="H37" s="9" t="n"/>
       <c r="I37" s="9" t="n"/>
-      <c r="AJ37" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
@@ -1426,11 +1241,6 @@
       <c r="G38" s="9" t="n"/>
       <c r="H38" s="9" t="n"/>
       <c r="I38" s="9" t="n"/>
-      <c r="AJ38" t="inlineStr">
-        <is>
-          <t>15:10</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
@@ -1446,11 +1256,6 @@
       <c r="G39" s="9" t="n"/>
       <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
-      <c r="AJ39" t="inlineStr">
-        <is>
-          <t>15:20</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
@@ -1466,11 +1271,6 @@
       <c r="G40" s="9" t="n"/>
       <c r="H40" s="9" t="n"/>
       <c r="I40" s="9" t="n"/>
-      <c r="AJ40" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
@@ -1486,11 +1286,6 @@
       <c r="G41" s="9" t="n"/>
       <c r="H41" s="9" t="n"/>
       <c r="I41" s="9" t="n"/>
-      <c r="AJ41" t="inlineStr">
-        <is>
-          <t>15:40</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
@@ -1506,11 +1301,6 @@
       <c r="G42" s="9" t="n"/>
       <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
-      <c r="AJ42" t="inlineStr">
-        <is>
-          <t>15:50</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
@@ -1526,11 +1316,6 @@
       <c r="G43" s="9" t="n"/>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
-      <c r="AJ43" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
@@ -1546,11 +1331,6 @@
       <c r="G44" s="9" t="n"/>
       <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
-      <c r="AJ44" t="inlineStr">
-        <is>
-          <t>16:10</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
@@ -1566,11 +1346,6 @@
       <c r="G45" s="9" t="n"/>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
-      <c r="AJ45" t="inlineStr">
-        <is>
-          <t>16:20</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
@@ -1586,11 +1361,6 @@
       <c r="G46" s="9" t="n"/>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
-      <c r="AJ46" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
@@ -1606,11 +1376,6 @@
       <c r="G47" s="9" t="n"/>
       <c r="H47" s="9" t="n"/>
       <c r="I47" s="9" t="n"/>
-      <c r="AJ47" t="inlineStr">
-        <is>
-          <t>16:40</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
@@ -1626,11 +1391,6 @@
       <c r="G48" s="9" t="n"/>
       <c r="H48" s="9" t="n"/>
       <c r="I48" s="9" t="n"/>
-      <c r="AJ48" t="inlineStr">
-        <is>
-          <t>16:50</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
@@ -1646,11 +1406,6 @@
       <c r="G49" s="9" t="n"/>
       <c r="H49" s="9" t="n"/>
       <c r="I49" s="9" t="n"/>
-      <c r="AJ49" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
@@ -1666,11 +1421,6 @@
       <c r="G50" s="9" t="n"/>
       <c r="H50" s="9" t="n"/>
       <c r="I50" s="9" t="n"/>
-      <c r="AJ50" t="inlineStr">
-        <is>
-          <t>17:10</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
@@ -1686,11 +1436,6 @@
       <c r="G51" s="9" t="n"/>
       <c r="H51" s="9" t="n"/>
       <c r="I51" s="9" t="n"/>
-      <c r="AJ51" t="inlineStr">
-        <is>
-          <t>17:20</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
@@ -1706,11 +1451,6 @@
       <c r="G52" s="9" t="n"/>
       <c r="H52" s="9" t="n"/>
       <c r="I52" s="9" t="n"/>
-      <c r="AJ52" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
@@ -1726,11 +1466,6 @@
       <c r="G53" s="9" t="n"/>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
-      <c r="AJ53" t="inlineStr">
-        <is>
-          <t>17:40</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
@@ -1746,11 +1481,6 @@
       <c r="G54" s="9" t="n"/>
       <c r="H54" s="9" t="n"/>
       <c r="I54" s="9" t="n"/>
-      <c r="AJ54" t="inlineStr">
-        <is>
-          <t>17:50</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
@@ -1766,11 +1496,6 @@
       <c r="G55" s="9" t="n"/>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
-      <c r="AJ55" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
@@ -1786,11 +1511,6 @@
       <c r="G56" s="9" t="n"/>
       <c r="H56" s="9" t="n"/>
       <c r="I56" s="9" t="n"/>
-      <c r="AJ56" t="inlineStr">
-        <is>
-          <t>18:10</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
@@ -1806,11 +1526,6 @@
       <c r="G57" s="9" t="n"/>
       <c r="H57" s="9" t="n"/>
       <c r="I57" s="9" t="n"/>
-      <c r="AJ57" t="inlineStr">
-        <is>
-          <t>18:20</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
@@ -1826,11 +1541,6 @@
       <c r="G58" s="9" t="n"/>
       <c r="H58" s="9" t="n"/>
       <c r="I58" s="9" t="n"/>
-      <c r="AJ58" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
@@ -2506,6 +2216,412 @@
       <c r="G103" s="9" t="n"/>
       <c r="H103" s="9" t="n"/>
       <c r="I103" s="9" t="n"/>
+    </row>
+    <row r="106">
+      <c r="AJ106" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="AJ107" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="AJ110" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="AJ111" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="AJ112" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="AJ115" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="AJ116" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="AJ117" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="AJ118" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="AJ119" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="AJ123" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="AJ124" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="AJ126" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="AJ128" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="AJ130" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="AJ131" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="AJ132" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="AJ133" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="AJ134" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="AJ135" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="AJ137" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="AJ139" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="AJ140" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="AJ141" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="AJ142" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="AJ143" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="AJ144" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="AJ145" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="AJ146" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>15:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="AJ148" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="AJ149" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="AJ150" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="AJ151" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="AJ152" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="AJ153" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="AJ154" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="AJ155" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="AJ156" t="inlineStr">
+        <is>
+          <t>17:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="AJ157" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="AJ158" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="AJ159" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="AJ160" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="AJ161" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="AJ162" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="AJ163" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2517,7 +2633,7 @@
       <formula1>"Tue 3 Nov,Wed 4 Nov,Thu 5 Nov,Fri 6 Nov"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:D103" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Time" error="Pick a time from the list." allowBlank="1" type="list">
-      <formula1>$AJ$1:$AJ$58</formula1>
+      <formula1>$AJ$106:$AJ$163</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F103" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Format" error="Pick a format from the list, or edit the list (Data validation) to add your own." allowBlank="1" type="list">
       <formula1>"AMA,Break,Closing,Demo,Fireside Chat,Fishbowl,Networking,Roundtable,Talk,Welcome,Workshop,Other"</formula1>

</xml_diff>

<commit_message>
Community Hubs: hourly live export of the hub sheets
- fileverse-live-export.yml reads every hub dSheet's live state (COMMUNITY_HUB_SHEETS secret) and commits devcon-api/data/community-hubs/sheets.json with [skip deploy]
- devcon-api reads that file from GitHub instead of Fileverse; COMMUNITY_HUB_SHEETS env no longer used
- Format "Break" rows are left out of the hubs bundle
- templates: visible, extendable time list in column K
</commit_message>
<xml_diff>
--- a/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
+++ b/devcon/public/community-hubs-templates/Agentic-Hub.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ163"/>
+  <dimension ref="A1:K183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="36" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -653,7 +653,7 @@
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col hidden="1" width="13" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2217,411 +2217,478 @@
       <c r="H103" s="9" t="n"/>
       <c r="I103" s="9" t="n"/>
     </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>Times for From/To: add more below</t>
+        </is>
+      </c>
+    </row>
     <row r="106">
-      <c r="AJ106" t="inlineStr">
+      <c r="K106" s="7" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="AJ107" t="inlineStr">
+      <c r="K107" s="7" t="inlineStr">
         <is>
           <t>09:10</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="AJ108" t="inlineStr">
+      <c r="K108" s="7" t="inlineStr">
         <is>
           <t>09:20</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="AJ109" t="inlineStr">
+      <c r="K109" s="7" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="AJ110" t="inlineStr">
+      <c r="K110" s="7" t="inlineStr">
         <is>
           <t>09:40</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="AJ111" t="inlineStr">
+      <c r="K111" s="7" t="inlineStr">
         <is>
           <t>09:50</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="AJ112" t="inlineStr">
+      <c r="K112" s="7" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="AJ113" t="inlineStr">
+      <c r="K113" s="7" t="inlineStr">
         <is>
           <t>10:10</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="AJ114" t="inlineStr">
+      <c r="K114" s="7" t="inlineStr">
         <is>
           <t>10:20</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="AJ115" t="inlineStr">
+      <c r="K115" s="7" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="AJ116" t="inlineStr">
+      <c r="K116" s="7" t="inlineStr">
         <is>
           <t>10:40</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="AJ117" t="inlineStr">
+      <c r="K117" s="7" t="inlineStr">
         <is>
           <t>10:50</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="AJ118" t="inlineStr">
+      <c r="K118" s="7" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="AJ119" t="inlineStr">
+      <c r="K119" s="7" t="inlineStr">
         <is>
           <t>11:10</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="AJ120" t="inlineStr">
+      <c r="K120" s="7" t="inlineStr">
         <is>
           <t>11:20</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="AJ121" t="inlineStr">
+      <c r="K121" s="7" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="AJ122" t="inlineStr">
+      <c r="K122" s="7" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="AJ123" t="inlineStr">
+      <c r="K123" s="7" t="inlineStr">
         <is>
           <t>11:50</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="AJ124" t="inlineStr">
+      <c r="K124" s="7" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="AJ125" t="inlineStr">
+      <c r="K125" s="7" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="AJ126" t="inlineStr">
+      <c r="K126" s="7" t="inlineStr">
         <is>
           <t>12:20</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="AJ127" t="inlineStr">
+      <c r="K127" s="7" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="AJ128" t="inlineStr">
+      <c r="K128" s="7" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="AJ129" t="inlineStr">
+      <c r="K129" s="7" t="inlineStr">
         <is>
           <t>12:50</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="AJ130" t="inlineStr">
+      <c r="K130" s="7" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="AJ131" t="inlineStr">
+      <c r="K131" s="7" t="inlineStr">
         <is>
           <t>13:10</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="AJ132" t="inlineStr">
+      <c r="K132" s="7" t="inlineStr">
         <is>
           <t>13:20</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="AJ133" t="inlineStr">
+      <c r="K133" s="7" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
     </row>
     <row r="134">
-      <c r="AJ134" t="inlineStr">
+      <c r="K134" s="7" t="inlineStr">
         <is>
           <t>13:40</t>
         </is>
       </c>
     </row>
     <row r="135">
-      <c r="AJ135" t="inlineStr">
+      <c r="K135" s="7" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="AJ136" t="inlineStr">
+      <c r="K136" s="7" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="AJ137" t="inlineStr">
+      <c r="K137" s="7" t="inlineStr">
         <is>
           <t>14:10</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="AJ138" t="inlineStr">
+      <c r="K138" s="7" t="inlineStr">
         <is>
           <t>14:20</t>
         </is>
       </c>
     </row>
     <row r="139">
-      <c r="AJ139" t="inlineStr">
+      <c r="K139" s="7" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
     </row>
     <row r="140">
-      <c r="AJ140" t="inlineStr">
+      <c r="K140" s="7" t="inlineStr">
         <is>
           <t>14:40</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="AJ141" t="inlineStr">
+      <c r="K141" s="7" t="inlineStr">
         <is>
           <t>14:50</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="AJ142" t="inlineStr">
+      <c r="K142" s="7" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="AJ143" t="inlineStr">
+      <c r="K143" s="7" t="inlineStr">
         <is>
           <t>15:10</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="AJ144" t="inlineStr">
+      <c r="K144" s="7" t="inlineStr">
         <is>
           <t>15:20</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="AJ145" t="inlineStr">
+      <c r="K145" s="7" t="inlineStr">
         <is>
           <t>15:30</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="AJ146" t="inlineStr">
+      <c r="K146" s="7" t="inlineStr">
         <is>
           <t>15:40</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="AJ147" t="inlineStr">
+      <c r="K147" s="7" t="inlineStr">
         <is>
           <t>15:50</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="AJ148" t="inlineStr">
+      <c r="K148" s="7" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="AJ149" t="inlineStr">
+      <c r="K149" s="7" t="inlineStr">
         <is>
           <t>16:10</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="AJ150" t="inlineStr">
+      <c r="K150" s="7" t="inlineStr">
         <is>
           <t>16:20</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="AJ151" t="inlineStr">
+      <c r="K151" s="7" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="AJ152" t="inlineStr">
+      <c r="K152" s="7" t="inlineStr">
         <is>
           <t>16:40</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="AJ153" t="inlineStr">
+      <c r="K153" s="7" t="inlineStr">
         <is>
           <t>16:50</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="AJ154" t="inlineStr">
+      <c r="K154" s="7" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="AJ155" t="inlineStr">
+      <c r="K155" s="7" t="inlineStr">
         <is>
           <t>17:10</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="AJ156" t="inlineStr">
+      <c r="K156" s="7" t="inlineStr">
         <is>
           <t>17:20</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="AJ157" t="inlineStr">
+      <c r="K157" s="7" t="inlineStr">
         <is>
           <t>17:30</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="AJ158" t="inlineStr">
+      <c r="K158" s="7" t="inlineStr">
         <is>
           <t>17:40</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="AJ159" t="inlineStr">
+      <c r="K159" s="7" t="inlineStr">
         <is>
           <t>17:50</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="AJ160" t="inlineStr">
+      <c r="K160" s="7" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="AJ161" t="inlineStr">
+      <c r="K161" s="7" t="inlineStr">
         <is>
           <t>18:10</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="AJ162" t="inlineStr">
+      <c r="K162" s="7" t="inlineStr">
         <is>
           <t>18:20</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="AJ163" t="inlineStr">
+      <c r="K163" s="7" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
+    </row>
+    <row r="164">
+      <c r="K164" s="7" t="n"/>
+    </row>
+    <row r="165">
+      <c r="K165" s="7" t="n"/>
+    </row>
+    <row r="166">
+      <c r="K166" s="7" t="n"/>
+    </row>
+    <row r="167">
+      <c r="K167" s="7" t="n"/>
+    </row>
+    <row r="168">
+      <c r="K168" s="7" t="n"/>
+    </row>
+    <row r="169">
+      <c r="K169" s="7" t="n"/>
+    </row>
+    <row r="170">
+      <c r="K170" s="7" t="n"/>
+    </row>
+    <row r="171">
+      <c r="K171" s="7" t="n"/>
+    </row>
+    <row r="172">
+      <c r="K172" s="7" t="n"/>
+    </row>
+    <row r="173">
+      <c r="K173" s="7" t="n"/>
+    </row>
+    <row r="174">
+      <c r="K174" s="7" t="n"/>
+    </row>
+    <row r="175">
+      <c r="K175" s="7" t="n"/>
+    </row>
+    <row r="176">
+      <c r="K176" s="7" t="n"/>
+    </row>
+    <row r="177">
+      <c r="K177" s="7" t="n"/>
+    </row>
+    <row r="178">
+      <c r="K178" s="7" t="n"/>
+    </row>
+    <row r="179">
+      <c r="K179" s="7" t="n"/>
+    </row>
+    <row r="180">
+      <c r="K180" s="7" t="n"/>
+    </row>
+    <row r="181">
+      <c r="K181" s="7" t="n"/>
+    </row>
+    <row r="182">
+      <c r="K182" s="7" t="n"/>
+    </row>
+    <row r="183">
+      <c r="K183" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2633,7 +2700,7 @@
       <formula1>"Tue 3 Nov,Wed 4 Nov,Thu 5 Nov,Fri 6 Nov"</formula1>
     </dataValidation>
     <dataValidation sqref="C4:D103" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Time" error="Pick a time from the list." allowBlank="1" type="list">
-      <formula1>$AJ$106:$AJ$163</formula1>
+      <formula1>$K$106:$K$183</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F103" showDropDown="0" showInputMessage="0" showErrorMessage="1" errorTitle="Format" error="Pick a format from the list, or edit the list (Data validation) to add your own." allowBlank="1" type="list">
       <formula1>"AMA,Break,Closing,Demo,Fireside Chat,Fishbowl,Networking,Roundtable,Talk,Welcome,Workshop,Other"</formula1>

</xml_diff>